<commit_message>
Apply pro-rata bulk allocations to 30th refund reconciliation
The three largest ETB orders (John Paulo Manuel 1000, Anton Canoy 850,
Vlade Mark Navarro 500) were carved out of the raffle and filled
pro-rata at 1.16%, yielding 12/10/6 units. Reconciles against total ETB
demand of 3,107 units. Reclassifies these rows from suspected data-entry
errors to confirmed bulk orders and flags their refunds for funds
verification before release.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Dak1TsnyGecM1Pgvoch9pH
</commit_message>
<xml_diff>
--- a/30th_Refund_List_RECONCILED.xlsx
+++ b/30th_Refund_List_RECONCILED.xlsx
@@ -170,8 +170,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1832,20 +1832,20 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="n">
+      <c r="A23" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Anton Canoy</t>
         </is>
       </c>
-      <c r="C23" s="8" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>PO-4CQ5ZZLJ</t>
         </is>
       </c>
-      <c r="D23" s="10" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>ETB x850</t>
         </is>
@@ -1853,25 +1853,29 @@
       <c r="E23" s="13" t="n">
         <v>850</v>
       </c>
-      <c r="F23" s="12" t="n">
+      <c r="F23" s="7" t="n">
         <v>1007250</v>
       </c>
       <c r="G23" s="14" t="n"/>
       <c r="H23" s="14" t="n">
         <v>1007250</v>
       </c>
-      <c r="I23" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J23" s="11" t="n"/>
-      <c r="K23" s="12" t="n"/>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>ETB x10</t>
+        </is>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K23" s="7" t="n">
+        <v>39500</v>
+      </c>
       <c r="L23" s="14" t="n">
-        <v>-1007250</v>
+        <v>-967750</v>
       </c>
       <c r="M23" s="14" t="n">
-        <v>1007250</v>
+        <v>967750</v>
       </c>
       <c r="N23" s="14" t="n"/>
       <c r="O23" s="15" t="inlineStr">
@@ -6124,20 +6128,20 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="n">
+      <c r="A93" s="4" t="n">
         <v>89</v>
       </c>
-      <c r="B93" s="8" t="inlineStr">
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>John Paulo Manuel</t>
         </is>
       </c>
-      <c r="C93" s="8" t="inlineStr">
+      <c r="C93" s="4" t="inlineStr">
         <is>
           <t>(none)</t>
         </is>
       </c>
-      <c r="D93" s="10" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>ETB x1000</t>
         </is>
@@ -6145,25 +6149,29 @@
       <c r="E93" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="F93" s="12" t="n">
+      <c r="F93" s="7" t="n">
         <v>1185000</v>
       </c>
       <c r="G93" s="14" t="n"/>
       <c r="H93" s="14" t="n">
         <v>1185000</v>
       </c>
-      <c r="I93" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J93" s="11" t="n"/>
-      <c r="K93" s="12" t="n"/>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>ETB x12</t>
+        </is>
+      </c>
+      <c r="J93" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="K93" s="7" t="n">
+        <v>47400</v>
+      </c>
       <c r="L93" s="14" t="n">
-        <v>-1185000</v>
+        <v>-1137600</v>
       </c>
       <c r="M93" s="14" t="n">
-        <v>1185000</v>
+        <v>1137600</v>
       </c>
       <c r="N93" s="14" t="n"/>
       <c r="O93" s="15" t="inlineStr">
@@ -10767,20 +10775,20 @@
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="8" t="n">
+      <c r="A170" s="4" t="n">
         <v>166</v>
       </c>
-      <c r="B170" s="8" t="inlineStr">
+      <c r="B170" s="4" t="inlineStr">
         <is>
           <t>Vlade Mark Navarro</t>
         </is>
       </c>
-      <c r="C170" s="8" t="inlineStr">
+      <c r="C170" s="4" t="inlineStr">
         <is>
           <t>Meta</t>
         </is>
       </c>
-      <c r="D170" s="10" t="inlineStr">
+      <c r="D170" s="5" t="inlineStr">
         <is>
           <t>ETB x500</t>
         </is>
@@ -10788,25 +10796,29 @@
       <c r="E170" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="F170" s="12" t="n">
+      <c r="F170" s="7" t="n">
         <v>592500</v>
       </c>
       <c r="G170" s="14" t="n"/>
       <c r="H170" s="14" t="n">
         <v>592500</v>
       </c>
-      <c r="I170" s="10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J170" s="11" t="n"/>
-      <c r="K170" s="12" t="n"/>
+      <c r="I170" s="5" t="inlineStr">
+        <is>
+          <t>ETB x6</t>
+        </is>
+      </c>
+      <c r="J170" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="K170" s="7" t="n">
+        <v>23700</v>
+      </c>
       <c r="L170" s="14" t="n">
-        <v>-592500</v>
+        <v>-568800</v>
       </c>
       <c r="M170" s="14" t="n">
-        <v>592500</v>
+        <v>568800</v>
       </c>
       <c r="N170" s="14" t="n"/>
       <c r="O170" s="15" t="inlineStr">
@@ -11124,7 +11136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -11154,7 +11166,7 @@
       </c>
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>Winner</t>
+          <t>Winner / Bulk Buyer</t>
         </is>
       </c>
       <c r="C3" s="19" t="inlineStr">
@@ -11206,37 +11218,37 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Renz Ryan Garcia</t>
+          <t>John Paulo Manuel</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>PO-EEJ5RN8E</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="D4" s="12" t="n">
         <v>3950</v>
       </c>
       <c r="E4" s="11" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F4" s="12" t="n">
-        <v>3950</v>
+        <v>47400</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>1185</v>
+        <v>1185000</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>2765</v>
+        <v>-1137600</v>
       </c>
       <c r="I4" s="20" t="inlineStr">
         <is>
-          <t>COLLECT ₱2,765.00</t>
-        </is>
-      </c>
-      <c r="J4" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+          <t>REFUND ₱1,137,600.00</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>BULK pro-rata 1.16% — ⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
@@ -11248,37 +11260,37 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Derick Valdez</t>
+          <t>Anton Canoy</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>PO-4MVMENX4</t>
+          <t>PO-4CQ5ZZLJ</t>
         </is>
       </c>
       <c r="D5" s="12" t="n">
         <v>3950</v>
       </c>
       <c r="E5" s="11" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F5" s="12" t="n">
-        <v>3950</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>4930</v>
-      </c>
-      <c r="H5" s="12" t="n">
-        <v>-980</v>
-      </c>
-      <c r="I5" s="8" t="inlineStr">
-        <is>
-          <t>REFUND ₱980.00</t>
-        </is>
-      </c>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>39500</v>
+      </c>
+      <c r="G5" s="14" t="n">
+        <v>1007250</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>-967750</v>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>REFUND ₱967,750.00</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>BULK pro-rata 1.16% — ⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
@@ -11290,37 +11302,37 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Rein Kevin Legarda</t>
+          <t>Vlade Mark Navarro</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>PO-V2VSTRHQ</t>
+          <t>Meta</t>
         </is>
       </c>
       <c r="D6" s="12" t="n">
         <v>3950</v>
       </c>
       <c r="E6" s="11" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F6" s="12" t="n">
-        <v>3950</v>
+        <v>23700</v>
       </c>
       <c r="G6" s="14" t="n">
-        <v>3330</v>
+        <v>592500</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>620</v>
+        <v>-568800</v>
       </c>
       <c r="I6" s="20" t="inlineStr">
         <is>
-          <t>COLLECT ₱620.00</t>
-        </is>
-      </c>
-      <c r="J6" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+          <t>REFUND ₱568,800.00</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>BULK pro-rata 1.16% — ⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
@@ -11332,12 +11344,12 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Albie Peralta</t>
+          <t>Renz Ryan Garcia</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>PO-VZ8HZ89W</t>
+          <t>PO-EEJ5RN8E</t>
         </is>
       </c>
       <c r="D7" s="12" t="n">
@@ -11349,20 +11361,20 @@
       <c r="F7" s="12" t="n">
         <v>3950</v>
       </c>
-      <c r="G7" s="12" t="n">
-        <v>6355</v>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>995</v>
-      </c>
-      <c r="I7" s="20" t="inlineStr">
-        <is>
-          <t>COLLECT ₱995.00</t>
-        </is>
-      </c>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="G7" s="14" t="n">
+        <v>1185</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>2765</v>
+      </c>
+      <c r="I7" s="21" t="inlineStr">
+        <is>
+          <t>COLLECT ₱2,765.00</t>
+        </is>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
@@ -11374,12 +11386,12 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>John David Laranang</t>
+          <t>Derick Valdez</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>PO-N8V8SM26</t>
+          <t>PO-4MVMENX4</t>
         </is>
       </c>
       <c r="D8" s="12" t="n">
@@ -11391,20 +11403,20 @@
       <c r="F8" s="12" t="n">
         <v>3950</v>
       </c>
-      <c r="G8" s="14" t="n">
-        <v>1185</v>
-      </c>
-      <c r="H8" s="14" t="n">
-        <v>2765</v>
-      </c>
-      <c r="I8" s="20" t="inlineStr">
-        <is>
-          <t>COLLECT ₱2,765.00</t>
-        </is>
-      </c>
-      <c r="J8" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+      <c r="G8" s="12" t="n">
+        <v>4930</v>
+      </c>
+      <c r="H8" s="12" t="n">
+        <v>-980</v>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>REFUND ₱980.00</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -11416,12 +11428,12 @@
       </c>
       <c r="B9" s="8" t="inlineStr">
         <is>
-          <t>Kris Becker</t>
+          <t>Rein Kevin Legarda</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>PO-E7CL8VNG</t>
+          <t>PO-V2VSTRHQ</t>
         </is>
       </c>
       <c r="D9" s="12" t="n">
@@ -11434,17 +11446,17 @@
         <v>3950</v>
       </c>
       <c r="G9" s="14" t="n">
-        <v>3045</v>
+        <v>3330</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>905</v>
-      </c>
-      <c r="I9" s="20" t="inlineStr">
-        <is>
-          <t>COLLECT ₱905.00</t>
-        </is>
-      </c>
-      <c r="J9" s="21" t="inlineStr">
+        <v>620</v>
+      </c>
+      <c r="I9" s="21" t="inlineStr">
+        <is>
+          <t>COLLECT ₱620.00</t>
+        </is>
+      </c>
+      <c r="J9" s="20" t="inlineStr">
         <is>
           <t>⚠ SFee not logged — provisional</t>
         </is>
@@ -11458,12 +11470,12 @@
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Francis Chen</t>
+          <t>Albie Peralta</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>PO-XTVZVR4B</t>
+          <t>PO-VZ8HZ89W</t>
         </is>
       </c>
       <c r="D10" s="12" t="n">
@@ -11476,14 +11488,14 @@
         <v>3950</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>1185</v>
+        <v>6355</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>2765</v>
-      </c>
-      <c r="I10" s="20" t="inlineStr">
-        <is>
-          <t>COLLECT ₱2,765.00</t>
+        <v>995</v>
+      </c>
+      <c r="I10" s="21" t="inlineStr">
+        <is>
+          <t>COLLECT ₱995.00</t>
         </is>
       </c>
       <c r="J10" s="8" t="inlineStr">
@@ -11495,40 +11507,40 @@
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Binder</t>
+          <t>ETB</t>
         </is>
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>maribel corpuz</t>
+          <t>John David Laranang</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>PO-3CS5Q9HN</t>
+          <t>PO-N8V8SM26</t>
         </is>
       </c>
       <c r="D11" s="12" t="n">
-        <v>2900</v>
+        <v>3950</v>
       </c>
       <c r="E11" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F11" s="12" t="n">
-        <v>2900</v>
+        <v>3950</v>
       </c>
       <c r="G11" s="14" t="n">
-        <v>3240</v>
+        <v>1185</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>-340</v>
+        <v>2765</v>
       </c>
       <c r="I11" s="21" t="inlineStr">
         <is>
-          <t>REFUND ₱340.00</t>
-        </is>
-      </c>
-      <c r="J11" s="21" t="inlineStr">
+          <t>COLLECT ₱2,765.00</t>
+        </is>
+      </c>
+      <c r="J11" s="20" t="inlineStr">
         <is>
           <t>⚠ SFee not logged — provisional</t>
         </is>
@@ -11537,247 +11549,247 @@
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Binder</t>
+          <t>ETB</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Gabriel Galang</t>
+          <t>Kris Becker</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>PO-4LL2XSE5</t>
+          <t>PO-E7CL8VNG</t>
         </is>
       </c>
       <c r="D12" s="12" t="n">
-        <v>2900</v>
+        <v>3950</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F12" s="12" t="n">
-        <v>2900</v>
-      </c>
-      <c r="G12" s="12" t="n">
-        <v>34170</v>
-      </c>
-      <c r="H12" s="12" t="n">
-        <v>-31270</v>
-      </c>
-      <c r="I12" s="8" t="inlineStr">
-        <is>
-          <t>REFUND ₱31,270.00</t>
-        </is>
-      </c>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>3950</v>
+      </c>
+      <c r="G12" s="14" t="n">
+        <v>3045</v>
+      </c>
+      <c r="H12" s="14" t="n">
+        <v>905</v>
+      </c>
+      <c r="I12" s="21" t="inlineStr">
+        <is>
+          <t>COLLECT ₱905.00</t>
+        </is>
+      </c>
+      <c r="J12" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Ex Tin 5107</t>
+          <t>ETB</t>
         </is>
       </c>
       <c r="B13" s="8" t="inlineStr">
         <is>
-          <t>Jomariz Hesita</t>
+          <t>Francis Chen</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>PO-V85HWE8A</t>
+          <t>PO-XTVZVR4B</t>
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>2000</v>
+        <v>3950</v>
       </c>
       <c r="E13" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F13" s="12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G13" s="14" t="n">
-        <v>8025</v>
-      </c>
-      <c r="H13" s="14" t="n">
-        <v>-6025</v>
+        <v>3950</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>1185</v>
+      </c>
+      <c r="H13" s="12" t="n">
+        <v>2765</v>
       </c>
       <c r="I13" s="21" t="inlineStr">
         <is>
-          <t>REFUND ₱6,025.00</t>
-        </is>
-      </c>
-      <c r="J13" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+          <t>COLLECT ₱2,765.00</t>
+        </is>
+      </c>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Ex Tin 5107</t>
+          <t>Binder</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Daisy Alvior</t>
+          <t>maribel corpuz</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>PO-KBPPLBNQ</t>
+          <t>PO-3CS5Q9HN</t>
         </is>
       </c>
       <c r="D14" s="12" t="n">
-        <v>2000</v>
+        <v>2900</v>
       </c>
       <c r="E14" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G14" s="12" t="n">
-        <v>5265</v>
-      </c>
-      <c r="H14" s="12" t="n">
-        <v>-3265</v>
-      </c>
-      <c r="I14" s="8" t="inlineStr">
-        <is>
-          <t>REFUND ₱3,265.00</t>
-        </is>
-      </c>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>2900</v>
+      </c>
+      <c r="G14" s="14" t="n">
+        <v>3240</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>-340</v>
+      </c>
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>REFUND ₱340.00</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Ex Tin 5107</t>
+          <t>Binder</t>
         </is>
       </c>
       <c r="B15" s="8" t="inlineStr">
         <is>
-          <t>Kerstie Dimple Barillo</t>
+          <t>Gabriel Galang</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>PO-82MFVCHZ</t>
+          <t>PO-4LL2XSE5</t>
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>2000</v>
+        <v>2900</v>
       </c>
       <c r="E15" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="12" t="n">
-        <v>2000</v>
-      </c>
-      <c r="G15" s="14" t="n">
-        <v>7305</v>
-      </c>
-      <c r="H15" s="14" t="n">
-        <v>-5305</v>
-      </c>
-      <c r="I15" s="21" t="inlineStr">
-        <is>
-          <t>REFUND ₱5,305.00</t>
-        </is>
-      </c>
-      <c r="J15" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+        <v>2900</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>34170</v>
+      </c>
+      <c r="H15" s="12" t="n">
+        <v>-31270</v>
+      </c>
+      <c r="I15" s="8" t="inlineStr">
+        <is>
+          <t>REFUND ₱31,270.00</t>
+        </is>
+      </c>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Sylveon Ex Box</t>
+          <t>Ex Tin 5107</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Albie Peralta</t>
+          <t>Jomariz Hesita</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>PO-VZ8HZ89W</t>
+          <t>PO-V85HWE8A</t>
         </is>
       </c>
       <c r="D16" s="12" t="n">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="E16" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="12" t="n">
-        <v>1800</v>
-      </c>
-      <c r="G16" s="12" t="n">
-        <v>6355</v>
-      </c>
-      <c r="H16" s="12" t="n">
-        <v>995</v>
+        <v>2000</v>
+      </c>
+      <c r="G16" s="14" t="n">
+        <v>8025</v>
+      </c>
+      <c r="H16" s="14" t="n">
+        <v>-6025</v>
       </c>
       <c r="I16" s="20" t="inlineStr">
         <is>
-          <t>COLLECT ₱995.00</t>
-        </is>
-      </c>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+          <t>REFUND ₱6,025.00</t>
+        </is>
+      </c>
+      <c r="J16" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Sylveon Ex Box</t>
+          <t>Ex Tin 5107</t>
         </is>
       </c>
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>Arianne Carranceja</t>
+          <t>Daisy Alvior</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
         <is>
-          <t>PO-GQSRTT8H</t>
+          <t>PO-KBPPLBNQ</t>
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="E17" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="12" t="n">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>26475</v>
+        <v>5265</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>-23075</v>
+        <v>-3265</v>
       </c>
       <c r="I17" s="8" t="inlineStr">
         <is>
-          <t>REFUND ₱23,075.00</t>
+          <t>REFUND ₱3,265.00</t>
         </is>
       </c>
       <c r="J17" s="8" t="inlineStr">
@@ -11789,40 +11801,40 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Sylveon Ex Box</t>
+          <t>Ex Tin 5107</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Leoflor Jimenez</t>
+          <t>Kerstie Dimple Barillo</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>PO-EF5WU62Y</t>
+          <t>PO-82MFVCHZ</t>
         </is>
       </c>
       <c r="D18" s="12" t="n">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="E18" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F18" s="12" t="n">
-        <v>1800</v>
+        <v>2000</v>
       </c>
       <c r="G18" s="14" t="n">
-        <v>2205</v>
+        <v>7305</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>-405</v>
-      </c>
-      <c r="I18" s="21" t="inlineStr">
-        <is>
-          <t>REFUND ₱405.00</t>
-        </is>
-      </c>
-      <c r="J18" s="21" t="inlineStr">
+        <v>-5305</v>
+      </c>
+      <c r="I18" s="20" t="inlineStr">
+        <is>
+          <t>REFUND ₱5,305.00</t>
+        </is>
+      </c>
+      <c r="J18" s="20" t="inlineStr">
         <is>
           <t>⚠ SFee not logged — provisional</t>
         </is>
@@ -11836,12 +11848,12 @@
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t>AL FRANCIS TESORERO</t>
+          <t>Albie Peralta</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
         <is>
-          <t>PO-59NFZENJ</t>
+          <t>PO-VZ8HZ89W</t>
         </is>
       </c>
       <c r="D19" s="12" t="n">
@@ -11854,14 +11866,14 @@
         <v>1800</v>
       </c>
       <c r="G19" s="12" t="n">
-        <v>7050</v>
+        <v>6355</v>
       </c>
       <c r="H19" s="12" t="n">
-        <v>-5250</v>
-      </c>
-      <c r="I19" s="8" t="inlineStr">
-        <is>
-          <t>REFUND ₱5,250.00</t>
+        <v>995</v>
+      </c>
+      <c r="I19" s="21" t="inlineStr">
+        <is>
+          <t>COLLECT ₱995.00</t>
         </is>
       </c>
       <c r="J19" s="8" t="inlineStr">
@@ -11873,37 +11885,37 @@
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sylveon Ex Box</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Albie Peralta</t>
+          <t>Arianne Carranceja</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>PO-VZ8HZ89W</t>
+          <t>PO-GQSRTT8H</t>
         </is>
       </c>
       <c r="D20" s="12" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="E20" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="12" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="G20" s="12" t="n">
-        <v>6355</v>
+        <v>26475</v>
       </c>
       <c r="H20" s="12" t="n">
-        <v>995</v>
-      </c>
-      <c r="I20" s="20" t="inlineStr">
-        <is>
-          <t>COLLECT ₱995.00</t>
+        <v>-23075</v>
+      </c>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>REFUND ₱23,075.00</t>
         </is>
       </c>
       <c r="J20" s="8" t="inlineStr">
@@ -11915,84 +11927,84 @@
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sylveon Ex Box</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t>Jared Chua</t>
+          <t>Leoflor Jimenez</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>PO-T24STP5E</t>
+          <t>PO-EF5WU62Y</t>
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="E21" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="12" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G21" s="12" t="n">
-        <v>6730</v>
-      </c>
-      <c r="H21" s="12" t="n">
-        <v>-5130</v>
-      </c>
-      <c r="I21" s="8" t="inlineStr">
-        <is>
-          <t>REFUND ₱5,130.00</t>
-        </is>
-      </c>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+        <v>1800</v>
+      </c>
+      <c r="G21" s="14" t="n">
+        <v>2205</v>
+      </c>
+      <c r="H21" s="14" t="n">
+        <v>-405</v>
+      </c>
+      <c r="I21" s="20" t="inlineStr">
+        <is>
+          <t>REFUND ₱405.00</t>
+        </is>
+      </c>
+      <c r="J21" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Poster</t>
+          <t>Sylveon Ex Box</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Michael Vivo</t>
+          <t>AL FRANCIS TESORERO</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>PO-MQ4V763G</t>
+          <t>PO-59NFZENJ</t>
         </is>
       </c>
       <c r="D22" s="12" t="n">
-        <v>1600</v>
+        <v>1800</v>
       </c>
       <c r="E22" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="12" t="n">
-        <v>1600</v>
-      </c>
-      <c r="G22" s="14" t="n">
-        <v>480</v>
-      </c>
-      <c r="H22" s="14" t="n">
-        <v>1120</v>
-      </c>
-      <c r="I22" s="20" t="inlineStr">
-        <is>
-          <t>COLLECT ₱1,120.00</t>
-        </is>
-      </c>
-      <c r="J22" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+        <v>1800</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>7050</v>
+      </c>
+      <c r="H22" s="12" t="n">
+        <v>-5250</v>
+      </c>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>REFUND ₱5,250.00</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -12004,12 +12016,12 @@
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>Joric Cabial</t>
+          <t>Albie Peralta</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>PO-TSYESURA</t>
+          <t>PO-VZ8HZ89W</t>
         </is>
       </c>
       <c r="D23" s="12" t="n">
@@ -12021,20 +12033,20 @@
       <c r="F23" s="12" t="n">
         <v>1600</v>
       </c>
-      <c r="G23" s="14" t="n">
-        <v>2520</v>
-      </c>
-      <c r="H23" s="14" t="n">
-        <v>-920</v>
+      <c r="G23" s="12" t="n">
+        <v>6355</v>
+      </c>
+      <c r="H23" s="12" t="n">
+        <v>995</v>
       </c>
       <c r="I23" s="21" t="inlineStr">
         <is>
-          <t>REFUND ₱920.00</t>
-        </is>
-      </c>
-      <c r="J23" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+          <t>COLLECT ₱995.00</t>
+        </is>
+      </c>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -12046,12 +12058,12 @@
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>MARK LAURENCE RECIO</t>
+          <t>Jared Chua</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>PO-BZ77X54L</t>
+          <t>PO-T24STP5E</t>
         </is>
       </c>
       <c r="D24" s="12" t="n">
@@ -12063,20 +12075,20 @@
       <c r="F24" s="12" t="n">
         <v>1600</v>
       </c>
-      <c r="G24" s="14" t="n">
-        <v>1350</v>
-      </c>
-      <c r="H24" s="14" t="n">
-        <v>250</v>
-      </c>
-      <c r="I24" s="20" t="inlineStr">
-        <is>
-          <t>COLLECT ₱250.00</t>
-        </is>
-      </c>
-      <c r="J24" s="21" t="inlineStr">
-        <is>
-          <t>⚠ SFee not logged — provisional</t>
+      <c r="G24" s="12" t="n">
+        <v>6730</v>
+      </c>
+      <c r="H24" s="12" t="n">
+        <v>-5130</v>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>REFUND ₱5,130.00</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
         </is>
       </c>
     </row>
@@ -12088,12 +12100,12 @@
       </c>
       <c r="B25" s="8" t="inlineStr">
         <is>
-          <t>Kim Saballegue</t>
+          <t>Michael Vivo</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>PO-QKUDKWFZ</t>
+          <t>PO-MQ4V763G</t>
         </is>
       </c>
       <c r="D25" s="12" t="n">
@@ -12106,17 +12118,17 @@
         <v>1600</v>
       </c>
       <c r="G25" s="14" t="n">
-        <v>9885</v>
+        <v>480</v>
       </c>
       <c r="H25" s="14" t="n">
-        <v>-6685</v>
+        <v>1120</v>
       </c>
       <c r="I25" s="21" t="inlineStr">
         <is>
-          <t>REFUND ₱6,685.00</t>
-        </is>
-      </c>
-      <c r="J25" s="21" t="inlineStr">
+          <t>COLLECT ₱1,120.00</t>
+        </is>
+      </c>
+      <c r="J25" s="20" t="inlineStr">
         <is>
           <t>⚠ SFee not logged — provisional</t>
         </is>
@@ -12130,12 +12142,12 @@
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Hannah Mariano</t>
+          <t>Joric Cabial</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>PO-E5CWZHPF</t>
+          <t>PO-TSYESURA</t>
         </is>
       </c>
       <c r="D26" s="12" t="n">
@@ -12147,37 +12159,37 @@
       <c r="F26" s="12" t="n">
         <v>1600</v>
       </c>
-      <c r="G26" s="12" t="n">
-        <v>29580</v>
-      </c>
-      <c r="H26" s="12" t="n">
-        <v>-26380</v>
-      </c>
-      <c r="I26" s="8" t="inlineStr">
-        <is>
-          <t>REFUND ₱26,380.00</t>
-        </is>
-      </c>
-      <c r="J26" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="G26" s="14" t="n">
+        <v>2520</v>
+      </c>
+      <c r="H26" s="14" t="n">
+        <v>-920</v>
+      </c>
+      <c r="I26" s="20" t="inlineStr">
+        <is>
+          <t>REFUND ₱920.00</t>
+        </is>
+      </c>
+      <c r="J26" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Tech Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
         <is>
-          <t>Arianne Carranceja</t>
+          <t>MARK LAURENCE RECIO</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>PO-GQSRTT8H</t>
+          <t>PO-BZ77X54L</t>
         </is>
       </c>
       <c r="D27" s="12" t="n">
@@ -12189,27 +12201,27 @@
       <c r="F27" s="12" t="n">
         <v>1600</v>
       </c>
-      <c r="G27" s="12" t="n">
-        <v>26475</v>
-      </c>
-      <c r="H27" s="12" t="n">
-        <v>-23075</v>
-      </c>
-      <c r="I27" s="8" t="inlineStr">
-        <is>
-          <t>REFUND ₱23,075.00</t>
-        </is>
-      </c>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>OK</t>
+      <c r="G27" s="14" t="n">
+        <v>1350</v>
+      </c>
+      <c r="H27" s="14" t="n">
+        <v>250</v>
+      </c>
+      <c r="I27" s="21" t="inlineStr">
+        <is>
+          <t>COLLECT ₱250.00</t>
+        </is>
+      </c>
+      <c r="J27" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Tech Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
@@ -12237,12 +12249,12 @@
       <c r="H28" s="14" t="n">
         <v>-6685</v>
       </c>
-      <c r="I28" s="21" t="inlineStr">
+      <c r="I28" s="20" t="inlineStr">
         <is>
           <t>REFUND ₱6,685.00</t>
         </is>
       </c>
-      <c r="J28" s="21" t="inlineStr">
+      <c r="J28" s="20" t="inlineStr">
         <is>
           <t>⚠ SFee not logged — provisional</t>
         </is>
@@ -12251,17 +12263,17 @@
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
         <is>
-          <t>Tech Sticker</t>
+          <t>Poster</t>
         </is>
       </c>
       <c r="B29" s="8" t="inlineStr">
         <is>
-          <t>Brandon Coyiuto</t>
+          <t>Hannah Mariano</t>
         </is>
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>PO-K6Z3RDEY</t>
+          <t>PO-E5CWZHPF</t>
         </is>
       </c>
       <c r="D29" s="12" t="n">
@@ -12274,14 +12286,14 @@
         <v>1600</v>
       </c>
       <c r="G29" s="12" t="n">
-        <v>24585</v>
+        <v>29580</v>
       </c>
       <c r="H29" s="12" t="n">
-        <v>-22985</v>
+        <v>-26380</v>
       </c>
       <c r="I29" s="8" t="inlineStr">
         <is>
-          <t>REFUND ₱22,985.00</t>
+          <t>REFUND ₱26,380.00</t>
         </is>
       </c>
       <c r="J29" s="8" t="inlineStr">
@@ -12298,12 +12310,12 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Hannah Mariano</t>
+          <t>Arianne Carranceja</t>
         </is>
       </c>
       <c r="C30" s="8" t="inlineStr">
         <is>
-          <t>PO-E5CWZHPF</t>
+          <t>PO-GQSRTT8H</t>
         </is>
       </c>
       <c r="D30" s="12" t="n">
@@ -12316,14 +12328,14 @@
         <v>1600</v>
       </c>
       <c r="G30" s="12" t="n">
-        <v>29580</v>
+        <v>26475</v>
       </c>
       <c r="H30" s="12" t="n">
-        <v>-26380</v>
+        <v>-23075</v>
       </c>
       <c r="I30" s="8" t="inlineStr">
         <is>
-          <t>REFUND ₱26,380.00</t>
+          <t>REFUND ₱23,075.00</t>
         </is>
       </c>
       <c r="J30" s="8" t="inlineStr">
@@ -12335,40 +12347,40 @@
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>2-Pack Blister</t>
+          <t>Tech Sticker</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>Louis Miguel Sta. Rita</t>
+          <t>Kim Saballegue</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>PO-QWTC3JJR</t>
+          <t>PO-QKUDKWFZ</t>
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>750</v>
+        <v>1600</v>
       </c>
       <c r="E31" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="12" t="n">
-        <v>750</v>
+        <v>1600</v>
       </c>
       <c r="G31" s="14" t="n">
-        <v>2820</v>
+        <v>9885</v>
       </c>
       <c r="H31" s="14" t="n">
-        <v>-2070</v>
-      </c>
-      <c r="I31" s="21" t="inlineStr">
-        <is>
-          <t>REFUND ₱2,070.00</t>
-        </is>
-      </c>
-      <c r="J31" s="21" t="inlineStr">
+        <v>-6685</v>
+      </c>
+      <c r="I31" s="20" t="inlineStr">
+        <is>
+          <t>REFUND ₱6,685.00</t>
+        </is>
+      </c>
+      <c r="J31" s="20" t="inlineStr">
         <is>
           <t>⚠ SFee not logged — provisional</t>
         </is>
@@ -12377,40 +12389,166 @@
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Knock Out</t>
+          <t>Tech Sticker</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Adrian Paul Baldonado</t>
+          <t>Brandon Coyiuto</t>
         </is>
       </c>
       <c r="C32" s="8" t="inlineStr">
         <is>
-          <t>PO-RADTSCLN</t>
+          <t>PO-K6Z3RDEY</t>
         </is>
       </c>
       <c r="D32" s="12" t="n">
-        <v>750</v>
+        <v>1600</v>
       </c>
       <c r="E32" s="11" t="n">
         <v>1</v>
       </c>
       <c r="F32" s="12" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G32" s="12" t="n">
+        <v>24585</v>
+      </c>
+      <c r="H32" s="12" t="n">
+        <v>-22985</v>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>REFUND ₱22,985.00</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>Tech Sticker</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Hannah Mariano</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>PO-E5CWZHPF</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E33" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="12" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G33" s="12" t="n">
+        <v>29580</v>
+      </c>
+      <c r="H33" s="12" t="n">
+        <v>-26380</v>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>REFUND ₱26,380.00</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>2-Pack Blister</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Louis Miguel Sta. Rita</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>PO-QWTC3JJR</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="n">
         <v>750</v>
       </c>
-      <c r="G32" s="12" t="n">
+      <c r="E34" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="12" t="n">
+        <v>750</v>
+      </c>
+      <c r="G34" s="14" t="n">
+        <v>2820</v>
+      </c>
+      <c r="H34" s="14" t="n">
+        <v>-2070</v>
+      </c>
+      <c r="I34" s="20" t="inlineStr">
+        <is>
+          <t>REFUND ₱2,070.00</t>
+        </is>
+      </c>
+      <c r="J34" s="20" t="inlineStr">
+        <is>
+          <t>⚠ SFee not logged — provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>Knock Out</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Adrian Paul Baldonado</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>PO-RADTSCLN</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="n">
+        <v>750</v>
+      </c>
+      <c r="E35" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="12" t="n">
+        <v>750</v>
+      </c>
+      <c r="G35" s="12" t="n">
         <v>2590</v>
       </c>
-      <c r="H32" s="12" t="n">
+      <c r="H35" s="12" t="n">
         <v>-1840</v>
       </c>
-      <c r="I32" s="8" t="inlineStr">
+      <c r="I35" s="8" t="inlineStr">
         <is>
           <t>REFUND ₱1,840.00</t>
         </is>
       </c>
-      <c r="J32" s="8" t="inlineStr">
+      <c r="J35" s="8" t="inlineStr">
         <is>
           <t>OK</t>
         </is>
@@ -15305,7 +15443,7 @@
       </c>
       <c r="B98" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C98" s="10" t="n">
@@ -15323,7 +15461,7 @@
       </c>
       <c r="F98" s="10" t="inlineStr">
         <is>
-          <t>Qty 80, DP ₱94,800.00. Confirm this is a real order.</t>
+          <t>Qty 80, DP ₱94,800.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15335,25 +15473,25 @@
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C99" s="10" t="n">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="D99" s="10" t="inlineStr">
         <is>
-          <t>Anton Canoy</t>
+          <t>Gabriel Galang</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>PO-4CQ5ZZLJ</t>
+          <t>PO-4LL2XSE5</t>
         </is>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>Qty 850, DP ₱1,007,250.00. Confirm this is a real order.</t>
+          <t>Qty 48, DP ₱33,870.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15365,25 +15503,25 @@
       </c>
       <c r="B100" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C100" s="10" t="n">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D100" s="10" t="inlineStr">
         <is>
-          <t>Gabriel Galang</t>
+          <t>Hannah Mariano</t>
         </is>
       </c>
       <c r="E100" s="10" t="inlineStr">
         <is>
-          <t>PO-4LL2XSE5</t>
+          <t>PO-E5CWZHPF</t>
         </is>
       </c>
       <c r="F100" s="10" t="inlineStr">
         <is>
-          <t>Qty 48, DP ₱33,870.00. Confirm this is a real order.</t>
+          <t>Qty 48, DP ₱29,520.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15395,25 +15533,25 @@
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C101" s="10" t="n">
-        <v>60</v>
+        <v>73</v>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>Hannah Mariano</t>
+          <t>Jared Chua</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>PO-E5CWZHPF</t>
+          <t>PO-7K297LTD</t>
         </is>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>Qty 48, DP ₱29,520.00. Confirm this is a real order.</t>
+          <t>Qty 50, DP ₱11,250.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15425,25 +15563,25 @@
       </c>
       <c r="B102" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C102" s="10" t="n">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>Jared Chua</t>
+          <t>Jervelyn Constantino</t>
         </is>
       </c>
       <c r="E102" s="10" t="inlineStr">
         <is>
-          <t>PO-7K297LTD</t>
+          <t>PO-9RWYWS9X</t>
         </is>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
-          <t>Qty 50, DP ₱11,250.00. Confirm this is a real order.</t>
+          <t>Qty 30, DP ₱35,550.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15455,25 +15593,25 @@
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C103" s="10" t="n">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>Jervelyn Constantino</t>
+          <t>Lawrence (Anti-Hero)</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>PO-9RWYWS9X</t>
+          <t>Meet</t>
         </is>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>Qty 30, DP ₱35,550.00. Confirm this is a real order.</t>
+          <t>Qty 120, DP ₱27,000.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15485,25 +15623,25 @@
       </c>
       <c r="B104" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C104" s="10" t="n">
-        <v>92</v>
+        <v>131</v>
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>John Paulo Manuel</t>
+          <t>Mark Puyales</t>
         </is>
       </c>
       <c r="E104" s="10" t="inlineStr">
         <is>
-          <t>(none)</t>
+          <t>PO-P3J3HDK4</t>
         </is>
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
-          <t>Qty 1000, DP ₱1,185,000.00. Confirm this is a real order.</t>
+          <t>Qty 50, DP ₱59,250.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15515,25 +15653,25 @@
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C105" s="10" t="n">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>Lawrence (Anti-Hero)</t>
+          <t>Marty Aw</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>Meet</t>
+          <t>PO-WBHBBGRR</t>
         </is>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>Qty 120, DP ₱27,000.00. Confirm this is a real order.</t>
+          <t>Qty 30, DP ₱35,550.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15545,25 +15683,25 @@
       </c>
       <c r="B106" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C106" s="10" t="n">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>Mark Puyales</t>
+          <t>Matthan Eurique Calabio</t>
         </is>
       </c>
       <c r="E106" s="10" t="inlineStr">
         <is>
-          <t>PO-P3J3HDK4</t>
+          <t>PO-ZZ72YGBF</t>
         </is>
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
-          <t>Qty 50, DP ₱59,250.00. Confirm this is a real order.</t>
+          <t>Qty 100, DP ₱118,500.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
@@ -15575,97 +15713,97 @@
       </c>
       <c r="B107" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Large order — raffle fill only</t>
         </is>
       </c>
       <c r="C107" s="10" t="n">
-        <v>133</v>
+        <v>148</v>
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>Marty Aw</t>
+          <t>Patrick Gan</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>PO-WBHBBGRR</t>
+          <t>PO-W4XC5YXX</t>
         </is>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t>Qty 30, DP ₱35,550.00. Confirm this is a real order.</t>
+          <t>Qty 50, DP ₱11,250.00. Received no pro-rata allocation; confirm none is owed.</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="24" t="inlineStr">
-        <is>
-          <t>VERIFY</t>
+      <c r="A108" s="15" t="inlineStr">
+        <is>
+          <t>BLOCKER</t>
         </is>
       </c>
       <c r="B108" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Very large refund — verify funds before release</t>
         </is>
       </c>
       <c r="C108" s="10" t="n">
-        <v>137</v>
+        <v>22</v>
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t>Matthan Eurique Calabio</t>
+          <t>Anton Canoy</t>
         </is>
       </c>
       <c r="E108" s="10" t="inlineStr">
         <is>
-          <t>PO-ZZ72YGBF</t>
+          <t>PO-4CQ5ZZLJ</t>
         </is>
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
-          <t>Qty 100, DP ₱118,500.00. Confirm this is a real order.</t>
+          <t>Pro-rata ETB x10 on 850 ordered. Refund ₱967,750.00. Confirm the ₱1,007,250.00 downpayment actually cleared and verify payee identity before releasing.</t>
         </is>
       </c>
     </row>
     <row r="109">
-      <c r="A109" s="24" t="inlineStr">
-        <is>
-          <t>VERIFY</t>
+      <c r="A109" s="15" t="inlineStr">
+        <is>
+          <t>BLOCKER</t>
         </is>
       </c>
       <c r="B109" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Very large refund — verify funds before release</t>
         </is>
       </c>
       <c r="C109" s="10" t="n">
-        <v>148</v>
+        <v>92</v>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>Patrick Gan</t>
+          <t>John Paulo Manuel</t>
         </is>
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>PO-W4XC5YXX</t>
+          <t>(none)</t>
         </is>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t>Qty 50, DP ₱11,250.00. Confirm this is a real order.</t>
+          <t>Pro-rata ETB x12 on 1000 ordered. Refund ₱1,137,600.00. Confirm the ₱1,185,000.00 downpayment actually cleared and verify payee identity before releasing.</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="24" t="inlineStr">
-        <is>
-          <t>VERIFY</t>
+      <c r="A110" s="15" t="inlineStr">
+        <is>
+          <t>BLOCKER</t>
         </is>
       </c>
       <c r="B110" s="10" t="inlineStr">
         <is>
-          <t>Bulk / possible data-entry error</t>
+          <t>Very large refund — verify funds before release</t>
         </is>
       </c>
       <c r="C110" s="10" t="n">
@@ -15683,7 +15821,7 @@
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
-          <t>Qty 500, DP ₱592,500.00. Confirm this is a real order.</t>
+          <t>Pro-rata ETB x6 on 500 ordered. Refund ₱568,800.00. Confirm the ₱592,500.00 downpayment actually cleared and verify payee identity before releasing.</t>
         </is>
       </c>
     </row>
@@ -16493,7 +16631,7 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
-          <t>Refund ₱1,007,250.00 owed but no bank/GCash recorded.</t>
+          <t>Refund ₱967,750.00 owed but no bank/GCash recorded.</t>
         </is>
       </c>
     </row>
@@ -18443,7 +18581,7 @@
       </c>
       <c r="F202" s="10" t="inlineStr">
         <is>
-          <t>Refund ₱1,185,000.00 owed but no bank/GCash recorded.</t>
+          <t>Refund ₱1,137,600.00 owed but no bank/GCash recorded.</t>
         </is>
       </c>
     </row>
@@ -20363,7 +20501,7 @@
       </c>
       <c r="F266" s="10" t="inlineStr">
         <is>
-          <t>Refund ₱592,500.00 owed but no bank/GCash recorded.</t>
+          <t>Refund ₱568,800.00 owed but no bank/GCash recorded.</t>
         </is>
       </c>
     </row>

</xml_diff>